<commit_message>
Physics loss formulatio using residual
</commit_message>
<xml_diff>
--- a/PINN_training_history.xlsx
+++ b/PINN_training_history.xlsx
@@ -413,61 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Lambda</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Epoch</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>NN_Loss</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Physics_Loss</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total_Loss</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Raw_Delta_Min</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Raw_Delta_Max</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Negative_Delta_Fraction</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Log10_Sigma_f</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Sigma_f</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
@@ -475,107 +445,87 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.001</v>
+        <v>34.99019241333008</v>
       </c>
       <c r="B2" t="n">
-        <v>1000</v>
+        <v>647.0714721679688</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06682328134775162</v>
+        <v>35.05490112304688</v>
       </c>
       <c r="D2" t="n">
-        <v>315.3790283203125</v>
+        <v>2.996006488800049</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3822023272514343</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-20.00064086914062</v>
-      </c>
-      <c r="G2" t="n">
-        <v>104.9770812988281</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.1684210598468781</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.8516833782196045</v>
-      </c>
-      <c r="J2" t="n">
-        <v>7.106951934061144</v>
-      </c>
-      <c r="K2" t="n">
-        <v>-0.1914098411798477</v>
+        <v>-0.10399129986763</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.01</v>
+        <v>34.62587356567383</v>
       </c>
       <c r="B3" t="n">
-        <v>1000</v>
+        <v>645.9072265625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.09687040001153946</v>
+        <v>35.27178192138672</v>
       </c>
       <c r="D3" t="n">
-        <v>310.3209838867188</v>
+        <v>2.996006488800049</v>
       </c>
       <c r="E3" t="n">
-        <v>3.200080156326294</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-20.00064086914062</v>
-      </c>
-      <c r="G3" t="n">
-        <v>104.9770812988281</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.1684210598468781</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.8516068458557129</v>
-      </c>
-      <c r="J3" t="n">
-        <v>7.105699641130048</v>
-      </c>
-      <c r="K3" t="n">
-        <v>-0.1913925111293793</v>
+        <v>-0.10399129986763</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.1</v>
+        <v>31.17437171936035</v>
       </c>
       <c r="B4" t="n">
-        <v>1000</v>
+        <v>634.309814453125</v>
       </c>
       <c r="C4" t="n">
-        <v>2.48803973197937</v>
+        <v>37.51747131347656</v>
       </c>
       <c r="D4" t="n">
-        <v>264.3735046386719</v>
+        <v>2.996006488800049</v>
       </c>
       <c r="E4" t="n">
-        <v>28.92539024353027</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-20.00064086914062</v>
-      </c>
-      <c r="G4" t="n">
-        <v>104.9770812988281</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.1684210598468781</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.8500487208366394</v>
-      </c>
-      <c r="J4" t="n">
-        <v>7.080252089385061</v>
-      </c>
-      <c r="K4" t="n">
-        <v>-0.1911052763462067</v>
+        <v>-0.1039913296699524</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1741.458740234375</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.1425862312316895</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1741.601318359375</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.99600625038147</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.1039917171001434</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>209076.265625</v>
+      </c>
+      <c r="B6" t="n">
+        <v>52317.74609375</v>
+      </c>
+      <c r="C6" t="n">
+        <v>732253.75</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.996005058288574</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.1039921492338181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>